<commit_message>
tools: update test_event_export_rows to merged parent logic
</commit_message>
<xml_diff>
--- a/exports/event_sample_export.xlsx
+++ b/exports/event_sample_export.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
   <si>
     <t>Task</t>
   </si>
@@ -49,19 +49,13 @@
     <t>Food &amp; Catering</t>
   </si>
   <si>
-    <t>Tea &amp; Coffee; Lunch</t>
-  </si>
-  <si>
-    <t>Eben</t>
-  </si>
-  <si>
-    <t>Tea &amp; Coffee</t>
-  </si>
-  <si>
-    <t>Snacks</t>
-  </si>
-  <si>
-    <t>Dinakar</t>
+    <t>Lunch; Snacks</t>
+  </si>
+  <si>
+    <t>Eben, Dinakar</t>
+  </si>
+  <si>
+    <t>» Tea &amp; Coffee</t>
   </si>
 </sst>
 </file>
@@ -449,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -549,7 +543,7 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E7" t="s">
         <v>9</v>
@@ -575,35 +569,12 @@
         <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
event-planner: merge assigned subtasks into parent export row
</commit_message>
<xml_diff>
--- a/exports/event_sample_export.xlsx
+++ b/exports/event_sample_export.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="14">
   <si>
     <t>Task</t>
   </si>
@@ -49,13 +49,10 @@
     <t>Food &amp; Catering</t>
   </si>
   <si>
-    <t>Lunch; Snacks</t>
+    <t>Lunch; Snacks; » Tea &amp; Coffee</t>
   </si>
   <si>
     <t>Eben, Dinakar</t>
-  </si>
-  <si>
-    <t>» Tea &amp; Coffee</t>
   </si>
 </sst>
 </file>
@@ -443,7 +440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
@@ -543,38 +540,15 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>